<commit_message>
SAVOLA corrected on the same growth-basis error
Its terminal was handed a profit figure, a depreciation charge and a working
capital balance ALL already grown by (1+g), which the sanctioned construction
grows again. Central 27.1153 -> 26.6424, gap -10.5% -> -12.1%.

The correction shows up in the ledger where it belongs: the terminal lever
read -0.6% and reads -2.3% corrected, so the route is 27.2426 -> 27.4379 ->
26.8054 -> 26.6424. It takes MORE off, not less.

Workbook, documents, register, figures, ledger and gap review all rebuilt on
it. Study checks: recalc 809 of 809 formula cells, 51 drivers, 30 tables 0
unreconciled, 383 prose figures 0 unmatched.

Four studies remain on this error: AIRARABIA, EMPOWER, DU, MODON.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017RcjXG4ETjADcoFJf123yY
</commit_message>
<xml_diff>
--- a/engine/savola_study/SAVOLA_Valuation_Model_19082026_public.xlsx
+++ b/engine/savola_study/SAVOLA_Valuation_Model_19082026_public.xlsx
@@ -3152,19 +3152,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>31.00501074795766</v>
+        <v>30.31657737936937</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>32.69578958564818</v>
+        <v>31.7163092725914</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>34.71778065477459</v>
+        <v>33.38299584873408</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>37.18914273816153</v>
+        <v>35.41187223926126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>40.29182376865352</v>
+        <v>37.9495871730258</v>
       </c>
     </row>
     <row r="7">
@@ -3174,19 +3174,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>26.55858376375969</v>
+        <v>25.94020240374591</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>27.77362240825633</v>
+        <v>26.90056858463738</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>29.1972344240047</v>
+        <v>28.01846231042661</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>30.89591974606553</v>
+        <v>29.34410845614482</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>32.96780979585585</v>
+        <v>30.95162195698432</v>
       </c>
     </row>
     <row r="8">
@@ -3196,19 +3196,19 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>22.78031358805377</v>
+        <v>22.22116499917403</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>23.64862124332247</v>
+        <v>22.86432087940199</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>24.64696135912883</v>
+        <v>23.59615647976344</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>25.81280966387594</v>
+        <v>24.44222955016812</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>27.1995731846445</v>
+        <v>25.43896268998162</v>
       </c>
     </row>
     <row r="9">
@@ -3218,19 +3218,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>19.53096562583809</v>
+        <v>19.02249414644142</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>20.14234917029902</v>
+        <v>19.43309851333283</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>20.8323436128443</v>
+        <v>19.88826107315428</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>21.62161910739921</v>
+        <v>20.39969807300299</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>22.53878873815317</v>
+        <v>20.98362796803861</v>
       </c>
     </row>
     <row r="10">
@@ -3240,19 +3240,19 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>16.70745198490754</v>
+        <v>16.24277756876086</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>17.12590555776576</v>
+        <v>16.48086774908405</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>17.58875096455754</v>
+        <v>16.73491713918488</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>18.1067200865888</v>
+        <v>17.00878393391331</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>18.6943072968628</v>
+        <v>17.30767897316629</v>
       </c>
     </row>
     <row r="12">
@@ -3279,7 +3279,7 @@
         <v>0.73</v>
       </c>
       <c r="B14" s="7" t="n">
-        <v>36.32992409657243</v>
+        <v>34.96485674624154</v>
       </c>
     </row>
     <row r="15">
@@ -3287,7 +3287,7 @@
         <v>0.9</v>
       </c>
       <c r="B15" s="7" t="n">
-        <v>30.12905407736743</v>
+        <v>28.93149129253096</v>
       </c>
     </row>
     <row r="16">
@@ -3295,7 +3295,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="7" t="n">
-        <v>27.05069765935827</v>
+        <v>25.93571991247888</v>
       </c>
     </row>
     <row r="17">
@@ -3303,7 +3303,7 @@
         <v>1.087</v>
       </c>
       <c r="B17" s="7" t="n">
-        <v>24.64696135912883</v>
+        <v>23.59615647976344</v>
       </c>
     </row>
     <row r="18">
@@ -3311,7 +3311,7 @@
         <v>1.2</v>
       </c>
       <c r="B18" s="7" t="n">
-        <v>21.84589621396383</v>
+        <v>20.86947414111219</v>
       </c>
     </row>
     <row r="19">
@@ -3319,7 +3319,7 @@
         <v>1.44</v>
       </c>
       <c r="B19" s="7" t="n">
-        <v>16.85278527665721</v>
+        <v>16.00768193112958</v>
       </c>
     </row>
     <row r="21">
@@ -3348,7 +3348,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>27.46646812286339</v>
+        <v>26.34036141098163</v>
       </c>
     </row>
     <row r="24">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>24.64696135912883</v>
+        <v>23.59615647976344</v>
       </c>
     </row>
     <row r="25">
@@ -3368,7 +3368,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>22.12278001195606</v>
+        <v>21.13902596103296</v>
       </c>
     </row>
   </sheetData>
@@ -4184,14 +4184,14 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>8.420918519369135</v>
+        <v>7.697414044414612</v>
       </c>
       <c r="C5" s="8">
         <f>DCF!C64</f>
         <v/>
       </c>
       <c r="D5" s="7" t="n">
-        <v>32.94953550907461</v>
+        <v>31.72730977748877</v>
       </c>
       <c r="E5" s="9">
         <f>Assumptions!$C$148</f>
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>18.44752455884244</v>
+        <v>17.52774214976238</v>
       </c>
       <c r="G11" s="11">
         <f>C11/$C$14-1</f>
@@ -4632,7 +4632,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>8.420918519369135</v>
+        <v>7.697414044414612</v>
       </c>
     </row>
     <row r="7">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>32.94953550907461</v>
+        <v>31.72730977748877</v>
       </c>
     </row>
     <row r="8">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>18.44752455884244</v>
+        <v>17.52774214976238</v>
       </c>
     </row>
     <row r="17">
@@ -4756,7 +4756,7 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>22.86246689780856</v>
+        <v>21.85910269010905</v>
       </c>
     </row>
     <row r="20">
@@ -4773,7 +4773,7 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>19.12211320925031</v>
+        <v>18.23056657362525</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
@@ -4783,7 +4783,7 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>24.18151312543466</v>
+        <v>23.1394732036656</v>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
@@ -4793,7 +4793,7 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>24.87757939973216</v>
+        <v>23.82077318388701</v>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
@@ -4803,7 +4803,7 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>22.81884204003903</v>
+        <v>21.81634134347257</v>
       </c>
     </row>
     <row r="26">
@@ -4931,10 +4931,10 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>27.46646812286339</v>
+        <v>26.34036141098163</v>
       </c>
       <c r="D34" s="7" t="n">
-        <v>22.12278001195606</v>
+        <v>21.13902596103296</v>
       </c>
     </row>
   </sheetData>
@@ -9023,22 +9023,22 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Terminal operating profit after tax (year five grown one year)</t>
+          <t>Year-five operating profit after tax (the perpetuity grows it once)</t>
         </is>
       </c>
       <c r="C24" s="30">
-        <f>F10*(1+C23)</f>
+        <f>F10</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Plus owned and intangible depreciation, grown one year (the right-of-use charge cancels out of this model's own free cash flow and is not added back here)</t>
+          <t>Plus owned and intangible depreciation (the right-of-use charge cancels out of this model's own free cash flow and is not added back here)</t>
         </is>
       </c>
       <c r="C25" s="30">
-        <f>740.0006883973025*(1+C23)</f>
+        <f>740.0006883973025</f>
         <v/>
       </c>
     </row>
@@ -9071,7 +9071,7 @@
         </is>
       </c>
       <c r="C28" s="30">
-        <f>-C22*5687.100743*(1+C23)</f>
+        <f>-C22*5687.100743</f>
         <v/>
       </c>
     </row>
@@ -9159,7 +9159,7 @@
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>22.81884204003903</v>
+        <v>21.81634134347257</v>
       </c>
     </row>
     <row r="38">
@@ -9443,7 +9443,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>CDS-basis fair value (engine re-run at the CDS-basis cost of capital; the CDS legs are the January-2026 vintage, flagged): SAR 22.86</t>
+          <t>CDS-basis fair value (engine re-run at the CDS-basis cost of capital; the CDS legs are the January-2026 vintage, flagged): SAR 21.86</t>
         </is>
       </c>
     </row>

</xml_diff>